<commit_message>
Limpieza final tras quitar el idioma del trabajador
Restos que se habían quedado atrás en el commit anterior:
- Privacidad.svelte: la política todavía listaba "idioma" como dato
  tratado del trabajador.
- ejemplos/trabajadores-ejemplo.xlsx: regenerado sin la columna "Idioma"
  (ya no se usa en el import).
- shared/src/constants.ts: IDIOMAS_MVP sin ningún uso en el repo (residuo
  de cuando ro/ar/fr no tenían traducción completa, terminada 2026-09-08).

CLAUDE.md actualizado. 167 tests, typecheck y build limpios en los 4
paquetes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011qjn7kqGuGh7ZGgVpjPkp6
</commit_message>
<xml_diff>
--- a/ejemplos/trabajadores-ejemplo.xlsx
+++ b/ejemplos/trabajadores-ejemplo.xlsx
@@ -31,28 +31,38 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <bgColor/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -61,13 +71,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -397,227 +409,191 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G9"/>
-  <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="8.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:F9"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" s="2" t="str">
         <v>Nombre</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" s="2" t="str">
         <v>Alias</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" s="2" t="str">
         <v>Cuadrilla</v>
       </c>
-      <c r="D1" t="str">
-        <v>Idioma</v>
-      </c>
-      <c r="E1" t="str">
+      <c r="D1" s="2" t="str">
         <v>Transporte</v>
       </c>
-      <c r="F1" t="str">
+      <c r="E1" s="2" t="str">
         <v>QR</v>
       </c>
-      <c r="G1" t="str">
+      <c r="F1" s="2" t="str">
         <v>Activo</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2" s="2" t="str">
         <v>Antonio Ramírez Soler</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B2" s="2" t="str">
         <v>ANTONIO</v>
       </c>
-      <c r="C2" t="str">
-        <v>Cuadrilla 1</v>
-      </c>
-      <c r="D2" t="str">
-        <v>es</v>
-      </c>
-      <c r="E2" t="str">
+      <c r="C2" s="2" t="str">
+        <v>Cuadrilla 1</v>
+      </c>
+      <c r="D2" s="2" t="str">
         <v>5,00</v>
       </c>
-      <c r="F2" t="str">
+      <c r="E2" s="2" t="str">
         <v>ANTONIO</v>
       </c>
-      <c r="G2" t="str">
+      <c r="F2" s="2" t="str">
         <v>sí</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3" s="2" t="str">
         <v>Carmen Ortega Ruiz</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B3" s="2" t="str">
         <v>CARMEN</v>
       </c>
-      <c r="C3" t="str">
-        <v>Cuadrilla 1</v>
-      </c>
-      <c r="D3" t="str">
-        <v>es</v>
-      </c>
-      <c r="E3" t="str">
+      <c r="C3" s="2" t="str">
+        <v>Cuadrilla 1</v>
+      </c>
+      <c r="D3" s="2" t="str">
         <v>5,00</v>
       </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
+      <c r="E3" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F3" s="2" t="str">
         <v>sí</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="A4" s="2" t="str">
         <v>Youssef El Amrani</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B4" s="2" t="str">
         <v>YOUSSEF</v>
       </c>
-      <c r="C4" t="str">
-        <v>Cuadrilla 1</v>
-      </c>
-      <c r="D4" t="str">
-        <v>ar</v>
-      </c>
-      <c r="E4" t="str">
+      <c r="C4" s="2" t="str">
+        <v>Cuadrilla 1</v>
+      </c>
+      <c r="D4" s="2" t="str">
         <v>4,50</v>
       </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
+      <c r="E4" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F4" s="2" t="str">
         <v>sí</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5" s="2" t="str">
         <v>Vasile Dumitru</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B5" s="2" t="str">
         <v>VASILE</v>
       </c>
-      <c r="C5" t="str">
-        <v>Cuadrilla 1</v>
-      </c>
-      <c r="D5" t="str">
-        <v>ro</v>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
+      <c r="C5" s="2" t="str">
+        <v>Cuadrilla 1</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="2" t="str">
         <v>sí</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
+      <c r="A6" s="2" t="str">
         <v>Adriana Stoica</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B6" s="2" t="str">
         <v>ADRIANA</v>
       </c>
-      <c r="C6" t="str">
-        <v>Cuadrilla 1</v>
-      </c>
-      <c r="D6" t="str">
-        <v>ro</v>
-      </c>
-      <c r="E6" t="str">
+      <c r="C6" s="2" t="str">
+        <v>Cuadrilla 1</v>
+      </c>
+      <c r="D6" s="2" t="str">
         <v>3,50</v>
       </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6" t="str">
+      <c r="E6" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F6" s="2" t="str">
         <v>no</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
+      <c r="A7" s="2" t="str">
         <v>Karim Haddad</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B7" s="2" t="str">
         <v>KARIM</v>
       </c>
-      <c r="C7" t="str">
-        <v>Cuadrilla 1</v>
-      </c>
-      <c r="D7" t="str">
-        <v>fr</v>
-      </c>
-      <c r="E7" t="str">
+      <c r="C7" s="2" t="str">
+        <v>Cuadrilla 1</v>
+      </c>
+      <c r="D7" s="2" t="str">
         <v>6,00</v>
       </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7" t="str">
+      <c r="E7" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="2" t="str">
         <v>sí</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
+      <c r="A8" s="2" t="str">
         <v>Rosa Molina Vega</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B8" s="2" t="str">
         <v>ROSA</v>
       </c>
-      <c r="C8" t="str">
-        <v>Cuadrilla 1</v>
-      </c>
-      <c r="D8" t="str">
-        <v>es</v>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
-        <v/>
-      </c>
-      <c r="G8" t="str">
+      <c r="C8" s="2" t="str">
+        <v>Cuadrilla 1</v>
+      </c>
+      <c r="D8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="2" t="str">
         <v>sí</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
+      <c r="A9" s="2" t="str">
         <v>Daniel Ionescu</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B9" s="2" t="str">
         <v>DANIEL</v>
       </c>
-      <c r="C9" t="str">
-        <v>Cuadrilla 1</v>
-      </c>
-      <c r="D9" t="str">
-        <v>en</v>
-      </c>
-      <c r="E9" t="str">
+      <c r="C9" s="2" t="str">
+        <v>Cuadrilla 1</v>
+      </c>
+      <c r="D9" s="2" t="str">
         <v>4,00</v>
       </c>
-      <c r="F9" t="str">
-        <v/>
-      </c>
-      <c r="G9" t="str">
+      <c r="E9" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F9" s="2" t="str">
         <v>sí</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>